<commit_message>
catálogo e importación con el modelo del EER corregido
- El producto se identifica por SKU (GET /productos/:sku) y la categoría
  es texto; se quitan id, estado y subcategorías
- El stock sale de catalogo.producto y nace en 0; se quita
  crearExistenciaSiFalta
- El motor de precios usa la tasa de impuesto de cada producto
- La importación guarda tasa_impuesto y codigo_item pasa a ser opcional
</commit_message>
<xml_diff>
--- a/apps/server/modules/admin/importacion/plantilla-de-productos.xlsx
+++ b/apps/server/modules/admin/importacion/plantilla-de-productos.xlsx
@@ -86,22 +86,22 @@
     <t>Descripción</t>
   </si>
   <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>texto</t>
+  </si>
+  <si>
+    <t>Código interno del ítem, por ejemplo PS5-001. El sistema no lo usa.</t>
+  </si>
+  <si>
     <t>Sí</t>
   </si>
   <si>
-    <t>texto</t>
-  </si>
-  <si>
-    <t>Código interno del ítem, por ejemplo PS5-001. El prefijo indica la subcategoría.</t>
-  </si>
-  <si>
     <t>Categoría del producto: Video Juegos, Legos, Trading Cards.</t>
   </si>
   <si>
     <t>Código único del producto. Si ya existe, la importación lo actualiza.</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>Descripción completa que ve el cliente.</t>
@@ -701,13 +701,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
         <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -715,13 +715,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
         <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -729,7 +729,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
         <v>25</v>
@@ -743,7 +743,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
         <v>25</v>
@@ -757,7 +757,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
         <v>32</v>
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
         <v>34</v>
@@ -813,7 +813,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>34</v>
@@ -841,7 +841,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
         <v>34</v>
@@ -869,7 +869,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
         <v>25</v>

</xml_diff>